<commit_message>
Atualização da base de produtos (excel)
</commit_message>
<xml_diff>
--- a/data/produtos.xlsx
+++ b/data/produtos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistemas\Pré-Atendimento\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0F7C3E-D647-4A39-9174-C913EFE5C6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58471B39-7358-43E0-B62D-666381B0F20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{4158BE41-1E8D-481E-AEE2-F0FC4BF443A8}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="100">
   <si>
     <t>nome</t>
   </si>
@@ -111,9 +111,6 @@
     <t>Pedra Rachão</t>
   </si>
   <si>
-    <t>int</t>
-  </si>
-  <si>
     <t>un</t>
   </si>
   <si>
@@ -129,23 +126,222 @@
     <t>Azulejo</t>
   </si>
   <si>
-    <t>Tinta Látex</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Tinta Acrílica</t>
-  </si>
-  <si>
-    <t>Tinta Esmalte</t>
+    <t>Brita 0</t>
+  </si>
+  <si>
+    <t>Pó de Pedra</t>
+  </si>
+  <si>
+    <t>Cascalho</t>
+  </si>
+  <si>
+    <t>Cimento e Argamassa</t>
+  </si>
+  <si>
+    <t>Cimento 50kg</t>
+  </si>
+  <si>
+    <t>Argamassa AC1 20kg</t>
+  </si>
+  <si>
+    <t>Argamassa AC2 20kg</t>
+  </si>
+  <si>
+    <t>Argamassa AC3 20kg</t>
+  </si>
+  <si>
+    <t>Rejunte 1kg</t>
+  </si>
+  <si>
+    <t>Rejunte 5kg</t>
+  </si>
+  <si>
+    <t>Tijolo Baiano</t>
+  </si>
+  <si>
+    <t>Canaleta de Concreto</t>
+  </si>
+  <si>
+    <t>Meio Bloco</t>
+  </si>
+  <si>
+    <t>Barra de Ferro 10mm</t>
+  </si>
+  <si>
+    <t>Barra de Ferro 12mm</t>
+  </si>
+  <si>
+    <t>Arame Recozido 1kg</t>
+  </si>
+  <si>
+    <t>Arame Farpado 500m</t>
+  </si>
+  <si>
+    <t>Tela Soldada</t>
+  </si>
+  <si>
+    <t>Prego 18x27 (kg)</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>Prego 17x21 (kg)</t>
+  </si>
+  <si>
+    <t>Ripa 5m</t>
+  </si>
+  <si>
+    <t>Tábua Pinus 3m</t>
+  </si>
+  <si>
+    <t>Compensado 10mm</t>
+  </si>
+  <si>
+    <t>Compensado 15mm</t>
+  </si>
+  <si>
+    <t>Cobertura</t>
+  </si>
+  <si>
+    <t>Telha Cerâmica</t>
+  </si>
+  <si>
+    <t>Telha Fibrocimento 2,44m</t>
+  </si>
+  <si>
+    <t>Telha Fibrocimento 3,05m</t>
+  </si>
+  <si>
+    <t>Cumeeira Fibrocimento</t>
+  </si>
+  <si>
+    <t>Manta Térmica</t>
+  </si>
+  <si>
+    <t>Prego Telheiro</t>
+  </si>
+  <si>
+    <t>Rodapé Cerâmico</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Gesso 40kg</t>
+  </si>
+  <si>
+    <t>Massa Corrida 25kg</t>
+  </si>
+  <si>
+    <t>Massa Acrílica 25kg</t>
+  </si>
+  <si>
+    <t>Selador 18L</t>
+  </si>
+  <si>
+    <t>Tinta Látex 18L</t>
+  </si>
+  <si>
+    <t>Tinta Acrílica 18L</t>
+  </si>
+  <si>
+    <t>Tinta Esmalte 3,6L</t>
+  </si>
+  <si>
+    <t>Verniz 3,6L</t>
+  </si>
+  <si>
+    <t>Thinner 5L</t>
+  </si>
+  <si>
+    <t>Rolo de Pintura</t>
+  </si>
+  <si>
+    <t>Pincel 2"</t>
+  </si>
+  <si>
+    <t>Bandeja de Pintura</t>
+  </si>
+  <si>
+    <t>Tubo PVC 25mm</t>
+  </si>
+  <si>
+    <t>Registro Esfera</t>
+  </si>
+  <si>
+    <t>Torneira Metal</t>
+  </si>
+  <si>
+    <t>Chuveiro Elétrico</t>
+  </si>
+  <si>
+    <t>Elétrica</t>
+  </si>
+  <si>
+    <t>Fio 2,5mm (100m)</t>
+  </si>
+  <si>
+    <t>Fio 4mm (100m)</t>
+  </si>
+  <si>
+    <t>Disjuntor 20A</t>
+  </si>
+  <si>
+    <t>Tomada Simples</t>
+  </si>
+  <si>
+    <t>Interruptor Simples</t>
+  </si>
+  <si>
+    <t>Lâmpada LED 12W</t>
+  </si>
+  <si>
+    <t>Quadro Distribuição</t>
+  </si>
+  <si>
+    <t>Ferramentas</t>
+  </si>
+  <si>
+    <t>Pá</t>
+  </si>
+  <si>
+    <t>Enxada</t>
+  </si>
+  <si>
+    <t>Colher de Pedreiro</t>
+  </si>
+  <si>
+    <t>Nível 60cm</t>
+  </si>
+  <si>
+    <t>Trena 5m</t>
+  </si>
+  <si>
+    <t>Marreta 2kg</t>
+  </si>
+  <si>
+    <t>Balde 20L</t>
+  </si>
+  <si>
+    <t>Carrinho de Mão</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,13 +367,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -490,11 +689,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22BA13D2-8BD4-4A6A-90F8-DD922486DCB7}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -521,7 +721,7 @@
       <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>120</v>
       </c>
       <c r="D2" t="s">
@@ -538,7 +738,7 @@
       <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>115</v>
       </c>
       <c r="D3" t="s">
@@ -553,10 +753,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4">
-        <v>140</v>
+        <v>33</v>
+      </c>
+      <c r="C4" s="1">
+        <v>135</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
@@ -570,10 +770,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5">
-        <v>145</v>
+        <v>25</v>
+      </c>
+      <c r="C5" s="1">
+        <v>140</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
@@ -587,10 +787,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6">
-        <v>150</v>
+        <v>26</v>
+      </c>
+      <c r="C6" s="1">
+        <v>145</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -601,257 +801,1243 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7">
-        <v>1.5</v>
+        <v>27</v>
+      </c>
+      <c r="C7" s="1">
+        <v>150</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8">
-        <v>4.5</v>
+        <v>34</v>
+      </c>
+      <c r="C8" s="1">
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9">
-        <v>6.5</v>
+        <v>35</v>
+      </c>
+      <c r="C9" s="1">
+        <v>100</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10">
-        <v>28</v>
+        <v>37</v>
+      </c>
+      <c r="C10" s="1">
+        <v>38</v>
       </c>
       <c r="D10" t="s">
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11">
-        <v>65</v>
+        <v>38</v>
+      </c>
+      <c r="C11" s="1">
+        <v>22</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12">
-        <v>30</v>
+        <v>39</v>
+      </c>
+      <c r="C12" s="1">
+        <v>28</v>
       </c>
       <c r="D12" t="s">
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13">
-        <v>180</v>
+        <v>40</v>
+      </c>
+      <c r="C13" s="1">
+        <v>35</v>
       </c>
       <c r="D13" t="s">
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14">
-        <v>220</v>
+        <v>41</v>
+      </c>
+      <c r="C14" s="1">
+        <v>6</v>
       </c>
       <c r="D14" t="s">
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15">
-        <v>95</v>
+        <v>42</v>
+      </c>
+      <c r="C15" s="1">
+        <v>22</v>
       </c>
       <c r="D15" t="s">
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16">
-        <v>28</v>
+        <v>5</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1.5</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17">
-        <v>45</v>
+        <v>43</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1.8</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18">
-        <v>22</v>
+        <v>6</v>
+      </c>
+      <c r="C18" s="1">
+        <v>4.5</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19">
-        <v>85</v>
+        <v>7</v>
+      </c>
+      <c r="C19" s="1">
+        <v>6.5</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20">
-        <v>18</v>
+        <v>44</v>
+      </c>
+      <c r="C20" s="1">
+        <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="1">
+        <v>28</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1">
+        <v>45</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="1">
+        <v>65</v>
+      </c>
+      <c r="D24" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="1">
+        <v>85</v>
+      </c>
+      <c r="D25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="1">
+        <v>18</v>
+      </c>
+      <c r="D26" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="1">
+        <v>450</v>
+      </c>
+      <c r="D27" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="1">
+        <v>180</v>
+      </c>
+      <c r="D28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="1">
+        <v>18</v>
+      </c>
+      <c r="D29" t="s">
+        <v>22</v>
+      </c>
+      <c r="E29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="1">
+        <v>17</v>
+      </c>
+      <c r="D30" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="1">
+        <v>22</v>
+      </c>
+      <c r="D31" t="s">
+        <v>22</v>
+      </c>
+      <c r="E31" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="1">
+        <v>12</v>
+      </c>
+      <c r="D32" t="s">
+        <v>22</v>
+      </c>
+      <c r="E32" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="1">
+        <v>85</v>
+      </c>
+      <c r="D33" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="1">
+        <v>35</v>
+      </c>
+      <c r="D34" t="s">
+        <v>22</v>
+      </c>
+      <c r="E34" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" t="s">
+        <v>56</v>
+      </c>
+      <c r="C35" s="1">
+        <v>120</v>
+      </c>
+      <c r="D35" t="s">
+        <v>22</v>
+      </c>
+      <c r="E35" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="1">
+        <v>160</v>
+      </c>
+      <c r="D36" t="s">
+        <v>22</v>
+      </c>
+      <c r="E36" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" t="s">
+        <v>59</v>
+      </c>
+      <c r="C37" s="1">
+        <v>2.8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>22</v>
+      </c>
+      <c r="E37" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" t="s">
+        <v>60</v>
+      </c>
+      <c r="C38" s="1">
+        <v>55</v>
+      </c>
+      <c r="D38" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" t="s">
+        <v>61</v>
+      </c>
+      <c r="C39" s="1">
+        <v>75</v>
+      </c>
+      <c r="D39" t="s">
+        <v>22</v>
+      </c>
+      <c r="E39" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" t="s">
+        <v>62</v>
+      </c>
+      <c r="C40" s="1">
+        <v>35</v>
+      </c>
+      <c r="D40" t="s">
+        <v>22</v>
+      </c>
+      <c r="E40" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" s="1">
+        <v>180</v>
+      </c>
+      <c r="D41" t="s">
+        <v>22</v>
+      </c>
+      <c r="E41" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" t="s">
+        <v>64</v>
+      </c>
+      <c r="C42" s="1">
+        <v>22</v>
+      </c>
+      <c r="D42" t="s">
+        <v>22</v>
+      </c>
+      <c r="E42" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" t="s">
+        <v>29</v>
+      </c>
+      <c r="C43" s="1">
+        <v>28</v>
+      </c>
+      <c r="D43" t="s">
+        <v>22</v>
+      </c>
+      <c r="E43" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" t="s">
+        <v>31</v>
+      </c>
+      <c r="C44" s="1">
+        <v>65</v>
+      </c>
+      <c r="D44" t="s">
+        <v>22</v>
+      </c>
+      <c r="E44" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="1">
+        <v>30</v>
+      </c>
+      <c r="D45" t="s">
+        <v>22</v>
+      </c>
+      <c r="E45" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" t="s">
+        <v>65</v>
+      </c>
+      <c r="C46" s="1">
+        <v>12</v>
+      </c>
+      <c r="D46" t="s">
+        <v>22</v>
+      </c>
+      <c r="E46" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>17</v>
+      </c>
+      <c r="B47" t="s">
+        <v>67</v>
+      </c>
+      <c r="C47" s="1">
+        <v>45</v>
+      </c>
+      <c r="D47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E47" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>17</v>
+      </c>
+      <c r="B48" t="s">
+        <v>68</v>
+      </c>
+      <c r="C48" s="1">
+        <v>65</v>
+      </c>
+      <c r="D48" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" t="s">
+        <v>69</v>
+      </c>
+      <c r="C49" s="1">
+        <v>85</v>
+      </c>
+      <c r="D49" t="s">
+        <v>22</v>
+      </c>
+      <c r="E49" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>17</v>
+      </c>
+      <c r="B50" t="s">
+        <v>70</v>
+      </c>
+      <c r="C50" s="1">
+        <v>120</v>
+      </c>
+      <c r="D50" t="s">
+        <v>22</v>
+      </c>
+      <c r="E50" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>18</v>
+      </c>
+      <c r="B51" t="s">
+        <v>71</v>
+      </c>
+      <c r="C51" s="1">
+        <v>180</v>
+      </c>
+      <c r="D51" t="s">
+        <v>22</v>
+      </c>
+      <c r="E51" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>18</v>
+      </c>
+      <c r="B52" t="s">
+        <v>72</v>
+      </c>
+      <c r="C52" s="1">
+        <v>220</v>
+      </c>
+      <c r="D52" t="s">
+        <v>22</v>
+      </c>
+      <c r="E52" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>18</v>
+      </c>
+      <c r="B53" t="s">
+        <v>73</v>
+      </c>
+      <c r="C53" s="1">
+        <v>95</v>
+      </c>
+      <c r="D53" t="s">
+        <v>22</v>
+      </c>
+      <c r="E53" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" t="s">
+        <v>74</v>
+      </c>
+      <c r="C54" s="1">
+        <v>110</v>
+      </c>
+      <c r="D54" t="s">
+        <v>22</v>
+      </c>
+      <c r="E54" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>18</v>
+      </c>
+      <c r="B55" t="s">
+        <v>75</v>
+      </c>
+      <c r="C55" s="1">
+        <v>75</v>
+      </c>
+      <c r="D55" t="s">
+        <v>22</v>
+      </c>
+      <c r="E55" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>18</v>
+      </c>
+      <c r="B56" t="s">
+        <v>76</v>
+      </c>
+      <c r="C56" s="1">
+        <v>18</v>
+      </c>
+      <c r="D56" t="s">
+        <v>22</v>
+      </c>
+      <c r="E56" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57" t="s">
+        <v>77</v>
+      </c>
+      <c r="C57" s="1">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
+        <v>22</v>
+      </c>
+      <c r="E57" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" t="s">
+        <v>78</v>
+      </c>
+      <c r="C58" s="1">
+        <v>15</v>
+      </c>
+      <c r="D58" t="s">
+        <v>22</v>
+      </c>
+      <c r="E58" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>14</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C59" s="1">
+        <v>18</v>
+      </c>
+      <c r="D59" t="s">
+        <v>22</v>
+      </c>
+      <c r="E59" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>14</v>
+      </c>
+      <c r="B60" t="s">
+        <v>79</v>
+      </c>
+      <c r="C60" s="1">
+        <v>22</v>
+      </c>
+      <c r="D60" t="s">
+        <v>22</v>
+      </c>
+      <c r="E60" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>14</v>
+      </c>
+      <c r="B61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C61" s="1">
+        <v>22</v>
+      </c>
+      <c r="D61" t="s">
+        <v>22</v>
+      </c>
+      <c r="E61" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>14</v>
+      </c>
+      <c r="B62" t="s">
         <v>16</v>
       </c>
-      <c r="C21">
+      <c r="C62" s="1">
         <v>320</v>
       </c>
-      <c r="D21" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" t="s">
-        <v>29</v>
+      <c r="D62" t="s">
+        <v>22</v>
+      </c>
+      <c r="E62" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>14</v>
+      </c>
+      <c r="B63" t="s">
+        <v>81</v>
+      </c>
+      <c r="C63" s="1">
+        <v>45</v>
+      </c>
+      <c r="D63" t="s">
+        <v>22</v>
+      </c>
+      <c r="E63" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>14</v>
+      </c>
+      <c r="B64" t="s">
+        <v>82</v>
+      </c>
+      <c r="C64" s="1">
+        <v>120</v>
+      </c>
+      <c r="D64" t="s">
+        <v>22</v>
+      </c>
+      <c r="E64" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>83</v>
+      </c>
+      <c r="B65" t="s">
+        <v>84</v>
+      </c>
+      <c r="C65" s="1">
+        <v>180</v>
+      </c>
+      <c r="D65" t="s">
+        <v>22</v>
+      </c>
+      <c r="E65" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>83</v>
+      </c>
+      <c r="B66" t="s">
+        <v>85</v>
+      </c>
+      <c r="C66" s="1">
+        <v>280</v>
+      </c>
+      <c r="D66" t="s">
+        <v>22</v>
+      </c>
+      <c r="E66" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>83</v>
+      </c>
+      <c r="B67" t="s">
+        <v>86</v>
+      </c>
+      <c r="C67" s="1">
+        <v>20</v>
+      </c>
+      <c r="D67" t="s">
+        <v>22</v>
+      </c>
+      <c r="E67" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>83</v>
+      </c>
+      <c r="B68" t="s">
+        <v>87</v>
+      </c>
+      <c r="C68" s="1">
+        <v>8</v>
+      </c>
+      <c r="D68" t="s">
+        <v>22</v>
+      </c>
+      <c r="E68" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>83</v>
+      </c>
+      <c r="B69" t="s">
+        <v>88</v>
+      </c>
+      <c r="C69" s="1">
+        <v>7</v>
+      </c>
+      <c r="D69" t="s">
+        <v>22</v>
+      </c>
+      <c r="E69" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>83</v>
+      </c>
+      <c r="B70" t="s">
+        <v>89</v>
+      </c>
+      <c r="C70" s="1">
+        <v>8</v>
+      </c>
+      <c r="D70" t="s">
+        <v>22</v>
+      </c>
+      <c r="E70" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>83</v>
+      </c>
+      <c r="B71" t="s">
+        <v>90</v>
+      </c>
+      <c r="C71" s="1">
+        <v>85</v>
+      </c>
+      <c r="D71" t="s">
+        <v>22</v>
+      </c>
+      <c r="E71" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>91</v>
+      </c>
+      <c r="B72" t="s">
+        <v>92</v>
+      </c>
+      <c r="C72" s="1">
+        <v>45</v>
+      </c>
+      <c r="D72" t="s">
+        <v>22</v>
+      </c>
+      <c r="E72" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>91</v>
+      </c>
+      <c r="B73" t="s">
+        <v>93</v>
+      </c>
+      <c r="C73" s="1">
+        <v>55</v>
+      </c>
+      <c r="D73" t="s">
+        <v>22</v>
+      </c>
+      <c r="E73" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>91</v>
+      </c>
+      <c r="B74" t="s">
+        <v>94</v>
+      </c>
+      <c r="C74" s="1">
+        <v>25</v>
+      </c>
+      <c r="D74" t="s">
+        <v>22</v>
+      </c>
+      <c r="E74" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>91</v>
+      </c>
+      <c r="B75" t="s">
+        <v>95</v>
+      </c>
+      <c r="C75" s="1">
+        <v>35</v>
+      </c>
+      <c r="D75" t="s">
+        <v>22</v>
+      </c>
+      <c r="E75" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>91</v>
+      </c>
+      <c r="B76" t="s">
+        <v>96</v>
+      </c>
+      <c r="C76" s="1">
+        <v>22</v>
+      </c>
+      <c r="D76" t="s">
+        <v>22</v>
+      </c>
+      <c r="E76" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>91</v>
+      </c>
+      <c r="B77" t="s">
+        <v>97</v>
+      </c>
+      <c r="C77" s="1">
+        <v>65</v>
+      </c>
+      <c r="D77" t="s">
+        <v>22</v>
+      </c>
+      <c r="E77" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>91</v>
+      </c>
+      <c r="B78" t="s">
+        <v>98</v>
+      </c>
+      <c r="C78" s="1">
+        <v>18</v>
+      </c>
+      <c r="D78" t="s">
+        <v>22</v>
+      </c>
+      <c r="E78" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>91</v>
+      </c>
+      <c r="B79" t="s">
+        <v>99</v>
+      </c>
+      <c r="C79" s="1">
+        <v>280</v>
+      </c>
+      <c r="D79" t="s">
+        <v>22</v>
+      </c>
+      <c r="E79" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização da base de produtos 2 (excel)
</commit_message>
<xml_diff>
--- a/data/produtos.xlsx
+++ b/data/produtos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistemas\Pré-Atendimento\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58471B39-7358-43E0-B62D-666381B0F20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F96AE2-AC8C-4E50-AA9C-8EEC8B8D79DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{4158BE41-1E8D-481E-AEE2-F0FC4BF443A8}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="91">
   <si>
     <t>nome</t>
   </si>
@@ -36,39 +36,6 @@
     <t>categoria</t>
   </si>
   <si>
-    <t>Agregados</t>
-  </si>
-  <si>
-    <t>Alvenaria</t>
-  </si>
-  <si>
-    <t>Tijolo Cerâmico</t>
-  </si>
-  <si>
-    <t>Bloco de Concreto 14x19x39</t>
-  </si>
-  <si>
-    <t>Bloco Estrutural</t>
-  </si>
-  <si>
-    <t>Ferragens</t>
-  </si>
-  <si>
-    <t>Barra de Ferro 6mm</t>
-  </si>
-  <si>
-    <t>Barra de Ferro 8mm</t>
-  </si>
-  <si>
-    <t>Madeira</t>
-  </si>
-  <si>
-    <t>Caibro 5x6</t>
-  </si>
-  <si>
-    <t>Viga 6m</t>
-  </si>
-  <si>
     <t>Hidráulica</t>
   </si>
   <si>
@@ -78,198 +45,24 @@
     <t>Caixa d'água 500L</t>
   </si>
   <si>
-    <t>Acabamento</t>
-  </si>
-  <si>
-    <t>Tintas</t>
-  </si>
-  <si>
     <t>tipo</t>
   </si>
   <si>
     <t>unidade</t>
   </si>
   <si>
-    <t>Areia Média</t>
-  </si>
-  <si>
     <t>decimal</t>
   </si>
   <si>
-    <t>m³</t>
-  </si>
-  <si>
-    <t>Areia Fina</t>
-  </si>
-  <si>
-    <t>Brita 1</t>
-  </si>
-  <si>
-    <t>Brita 2</t>
-  </si>
-  <si>
-    <t>Pedra Rachão</t>
-  </si>
-  <si>
     <t>un</t>
   </si>
   <si>
-    <t>Piso Cerâmico</t>
-  </si>
-  <si>
-    <t>m²</t>
-  </si>
-  <si>
-    <t>Porcelanato</t>
-  </si>
-  <si>
-    <t>Azulejo</t>
-  </si>
-  <si>
-    <t>Brita 0</t>
-  </si>
-  <si>
-    <t>Pó de Pedra</t>
-  </si>
-  <si>
-    <t>Cascalho</t>
-  </si>
-  <si>
-    <t>Cimento e Argamassa</t>
-  </si>
-  <si>
-    <t>Cimento 50kg</t>
-  </si>
-  <si>
-    <t>Argamassa AC1 20kg</t>
-  </si>
-  <si>
-    <t>Argamassa AC2 20kg</t>
-  </si>
-  <si>
-    <t>Argamassa AC3 20kg</t>
-  </si>
-  <si>
-    <t>Rejunte 1kg</t>
-  </si>
-  <si>
-    <t>Rejunte 5kg</t>
-  </si>
-  <si>
-    <t>Tijolo Baiano</t>
-  </si>
-  <si>
-    <t>Canaleta de Concreto</t>
-  </si>
-  <si>
-    <t>Meio Bloco</t>
-  </si>
-  <si>
-    <t>Barra de Ferro 10mm</t>
-  </si>
-  <si>
-    <t>Barra de Ferro 12mm</t>
-  </si>
-  <si>
-    <t>Arame Recozido 1kg</t>
-  </si>
-  <si>
-    <t>Arame Farpado 500m</t>
-  </si>
-  <si>
-    <t>Tela Soldada</t>
-  </si>
-  <si>
-    <t>Prego 18x27 (kg)</t>
-  </si>
-  <si>
-    <t>kg</t>
-  </si>
-  <si>
-    <t>Prego 17x21 (kg)</t>
-  </si>
-  <si>
-    <t>Ripa 5m</t>
-  </si>
-  <si>
-    <t>Tábua Pinus 3m</t>
-  </si>
-  <si>
-    <t>Compensado 10mm</t>
-  </si>
-  <si>
-    <t>Compensado 15mm</t>
-  </si>
-  <si>
-    <t>Cobertura</t>
-  </si>
-  <si>
-    <t>Telha Cerâmica</t>
-  </si>
-  <si>
-    <t>Telha Fibrocimento 2,44m</t>
-  </si>
-  <si>
-    <t>Telha Fibrocimento 3,05m</t>
-  </si>
-  <si>
-    <t>Cumeeira Fibrocimento</t>
-  </si>
-  <si>
-    <t>Manta Térmica</t>
-  </si>
-  <si>
-    <t>Prego Telheiro</t>
-  </si>
-  <si>
-    <t>Rodapé Cerâmico</t>
-  </si>
-  <si>
     <t>m</t>
   </si>
   <si>
-    <t>Gesso 40kg</t>
-  </si>
-  <si>
-    <t>Massa Corrida 25kg</t>
-  </si>
-  <si>
-    <t>Massa Acrílica 25kg</t>
-  </si>
-  <si>
-    <t>Selador 18L</t>
-  </si>
-  <si>
-    <t>Tinta Látex 18L</t>
-  </si>
-  <si>
-    <t>Tinta Acrílica 18L</t>
-  </si>
-  <si>
-    <t>Tinta Esmalte 3,6L</t>
-  </si>
-  <si>
-    <t>Verniz 3,6L</t>
-  </si>
-  <si>
-    <t>Thinner 5L</t>
-  </si>
-  <si>
-    <t>Rolo de Pintura</t>
-  </si>
-  <si>
-    <t>Pincel 2"</t>
-  </si>
-  <si>
-    <t>Bandeja de Pintura</t>
-  </si>
-  <si>
     <t>Tubo PVC 25mm</t>
   </si>
   <si>
-    <t>Registro Esfera</t>
-  </si>
-  <si>
     <t>Torneira Metal</t>
   </si>
   <si>
@@ -279,12 +72,6 @@
     <t>Elétrica</t>
   </si>
   <si>
-    <t>Fio 2,5mm (100m)</t>
-  </si>
-  <si>
-    <t>Fio 4mm (100m)</t>
-  </si>
-  <si>
     <t>Disjuntor 20A</t>
   </si>
   <si>
@@ -297,51 +84,227 @@
     <t>Lâmpada LED 12W</t>
   </si>
   <si>
-    <t>Quadro Distribuição</t>
-  </si>
-  <si>
-    <t>Ferramentas</t>
-  </si>
-  <si>
-    <t>Pá</t>
-  </si>
-  <si>
-    <t>Enxada</t>
-  </si>
-  <si>
-    <t>Colher de Pedreiro</t>
-  </si>
-  <si>
-    <t>Nível 60cm</t>
-  </si>
-  <si>
-    <t>Trena 5m</t>
-  </si>
-  <si>
-    <t>Marreta 2kg</t>
-  </si>
-  <si>
-    <t>Balde 20L</t>
-  </si>
-  <si>
-    <t>Carrinho de Mão</t>
+    <t>Tubo PVC 32mm</t>
+  </si>
+  <si>
+    <t>Tubo PVC 40mm</t>
+  </si>
+  <si>
+    <t>Tubo PVC 50mm</t>
+  </si>
+  <si>
+    <t>Joelho 90° 20mm</t>
+  </si>
+  <si>
+    <t>Joelho 90° 25mm</t>
+  </si>
+  <si>
+    <t>Joelho 90° 32mm</t>
+  </si>
+  <si>
+    <t>Tê 20mm</t>
+  </si>
+  <si>
+    <t>Tê 25mm</t>
+  </si>
+  <si>
+    <t>Tê 32mm</t>
+  </si>
+  <si>
+    <t>Registro Esfera 20mm</t>
+  </si>
+  <si>
+    <t>Registro Esfera 25mm</t>
+  </si>
+  <si>
+    <t>Registro Gaveta 25mm</t>
+  </si>
+  <si>
+    <t>Registro Pressão 20mm</t>
+  </si>
+  <si>
+    <t>Adaptador 20mm</t>
+  </si>
+  <si>
+    <t>Adaptador 25mm</t>
+  </si>
+  <si>
+    <t>Luva PVC 20mm</t>
+  </si>
+  <si>
+    <t>Luva PVC 25mm</t>
+  </si>
+  <si>
+    <t>Caixa d'água 1000L</t>
+  </si>
+  <si>
+    <t>Torneira Plástica</t>
+  </si>
+  <si>
+    <t>Chuveiro Simples</t>
+  </si>
+  <si>
+    <t>Sifão Sanfonado</t>
+  </si>
+  <si>
+    <t>Válvula Pia</t>
+  </si>
+  <si>
+    <t>Caixa Sifonada</t>
+  </si>
+  <si>
+    <t>Ralo Simples</t>
+  </si>
+  <si>
+    <t>Ralo Inox</t>
+  </si>
+  <si>
+    <t>Mangueira Jardim 20m</t>
+  </si>
+  <si>
+    <t>Mangueira Jardim 30m</t>
+  </si>
+  <si>
+    <t>Engate Flexível 40cm</t>
+  </si>
+  <si>
+    <t>Engate Flexível 60cm</t>
+  </si>
+  <si>
+    <t>Fita Veda Rosca</t>
+  </si>
+  <si>
+    <t>Cola PVC 175g</t>
+  </si>
+  <si>
+    <t>Cola PVC 850g</t>
+  </si>
+  <si>
+    <t>Caixa de Gordura</t>
+  </si>
+  <si>
+    <t>Caixa de Inspeção</t>
+  </si>
+  <si>
+    <t>Fio 1,5mm (rolo 100m)</t>
+  </si>
+  <si>
+    <t>Fio 2,5mm (rolo 100m)</t>
+  </si>
+  <si>
+    <t>Fio 4mm (rolo 100m)</t>
+  </si>
+  <si>
+    <t>Fio 6mm (rolo 100m)</t>
+  </si>
+  <si>
+    <t>Cabo PP 2x1,5mm</t>
+  </si>
+  <si>
+    <t>Cabo PP 2x2,5mm</t>
+  </si>
+  <si>
+    <t>Disjuntor 10A</t>
+  </si>
+  <si>
+    <t>Disjuntor 16A</t>
+  </si>
+  <si>
+    <t>Disjuntor 32A</t>
+  </si>
+  <si>
+    <t>Disjuntor 50A</t>
+  </si>
+  <si>
+    <t>Quadro de Distribuição 6 disjuntores</t>
+  </si>
+  <si>
+    <t>Quadro de Distribuição 12 disjuntores</t>
+  </si>
+  <si>
+    <t>Tomada Dupla</t>
+  </si>
+  <si>
+    <t>Interruptor Duplo</t>
+  </si>
+  <si>
+    <t>Interruptor Triplo</t>
+  </si>
+  <si>
+    <t>Espelho 1 módulo</t>
+  </si>
+  <si>
+    <t>Espelho 2 módulos</t>
+  </si>
+  <si>
+    <t>Espelho 3 módulos</t>
+  </si>
+  <si>
+    <t>Lâmpada LED 9W</t>
+  </si>
+  <si>
+    <t>Lâmpada LED 15W</t>
+  </si>
+  <si>
+    <t>Lâmpada LED 20W</t>
+  </si>
+  <si>
+    <t>Refletor LED 50W</t>
+  </si>
+  <si>
+    <t>Refletor LED 100W</t>
+  </si>
+  <si>
+    <t>Soquete E27</t>
+  </si>
+  <si>
+    <t>Extensão 5m</t>
+  </si>
+  <si>
+    <t>Extensão 10m</t>
+  </si>
+  <si>
+    <t>Fita Isolante</t>
+  </si>
+  <si>
+    <t>Conector Wago (kit)</t>
+  </si>
+  <si>
+    <t>Caixa de Luz 4x2</t>
+  </si>
+  <si>
+    <t>Caixa de Luz 4x4</t>
+  </si>
+  <si>
+    <t>Eletroduto 20mm</t>
+  </si>
+  <si>
+    <t>Eletroduto 25mm</t>
+  </si>
+  <si>
+    <t>Curva Eletroduto</t>
+  </si>
+  <si>
+    <t>Abraçadeira Nylon (100un)</t>
+  </si>
+  <si>
+    <t>Relé Fotocélula</t>
+  </si>
+  <si>
+    <t>Campainha Residencial</t>
+  </si>
+  <si>
+    <t>Transformador 127/220</t>
+  </si>
+  <si>
+    <t>int</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -367,16 +330,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -689,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22BA13D2-8BD4-4A6A-90F8-DD922486DCB7}">
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -708,10 +668,10 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -719,16 +679,16 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="1">
-        <v>120</v>
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -736,16 +696,16 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="1">
-        <v>115</v>
+        <v>11</v>
+      </c>
+      <c r="C3">
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -753,16 +713,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="1">
-        <v>135</v>
+        <v>19</v>
+      </c>
+      <c r="C4">
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -770,16 +730,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="1">
-        <v>140</v>
+        <v>20</v>
+      </c>
+      <c r="C5">
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -787,16 +747,16 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="1">
-        <v>145</v>
+        <v>21</v>
+      </c>
+      <c r="C6">
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -804,16 +764,16 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="1">
-        <v>150</v>
+        <v>22</v>
+      </c>
+      <c r="C7">
+        <v>2.5</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -821,16 +781,16 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="1">
-        <v>110</v>
+        <v>23</v>
+      </c>
+      <c r="C8">
+        <v>3.5</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -838,849 +798,849 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="1">
-        <v>100</v>
+        <v>24</v>
+      </c>
+      <c r="C9">
+        <v>4.5</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="1">
-        <v>38</v>
+        <v>25</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E10" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="1">
-        <v>22</v>
+        <v>26</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="1">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>5.5</v>
       </c>
       <c r="D12" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="1">
-        <v>35</v>
+        <v>28</v>
+      </c>
+      <c r="C13">
+        <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="1">
-        <v>6</v>
+        <v>29</v>
+      </c>
+      <c r="C14">
+        <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="1">
-        <v>22</v>
+        <v>30</v>
+      </c>
+      <c r="C15">
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="1">
-        <v>1.5</v>
+        <v>31</v>
+      </c>
+      <c r="C16">
+        <v>28</v>
       </c>
       <c r="D16" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="1">
-        <v>1.8</v>
+        <v>32</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E17" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" s="1">
-        <v>4.5</v>
+        <v>33</v>
+      </c>
+      <c r="C18">
+        <v>2.5</v>
       </c>
       <c r="D18" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E18" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="1">
-        <v>6.5</v>
+        <v>34</v>
+      </c>
+      <c r="C19">
+        <v>1.8</v>
       </c>
       <c r="D19" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E19" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="1">
-        <v>7</v>
+        <v>35</v>
+      </c>
+      <c r="C20">
+        <v>2.5</v>
       </c>
       <c r="D20" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E20" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21" s="1">
-        <v>3.5</v>
+        <v>5</v>
+      </c>
+      <c r="C21">
+        <v>320</v>
       </c>
       <c r="D21" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E21" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="1">
-        <v>28</v>
+        <v>36</v>
+      </c>
+      <c r="C22">
+        <v>580</v>
       </c>
       <c r="D22" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E22" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" s="1">
-        <v>45</v>
+        <v>37</v>
+      </c>
+      <c r="C23">
+        <v>15</v>
       </c>
       <c r="D23" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E23" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="1">
-        <v>65</v>
+        <v>12</v>
+      </c>
+      <c r="C24">
+        <v>45</v>
       </c>
       <c r="D24" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E24" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" s="1">
-        <v>85</v>
+        <v>38</v>
+      </c>
+      <c r="C25">
+        <v>35</v>
       </c>
       <c r="D25" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E25" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>48</v>
-      </c>
-      <c r="C26" s="1">
-        <v>18</v>
+        <v>13</v>
+      </c>
+      <c r="C26">
+        <v>120</v>
       </c>
       <c r="D26" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E26" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>49</v>
-      </c>
-      <c r="C27" s="1">
-        <v>450</v>
+        <v>39</v>
+      </c>
+      <c r="C27">
+        <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E27" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="1">
-        <v>180</v>
+        <v>40</v>
+      </c>
+      <c r="C28">
+        <v>10</v>
       </c>
       <c r="D28" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E28" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C29" s="1">
-        <v>18</v>
+        <v>41</v>
+      </c>
+      <c r="C29">
+        <v>25</v>
       </c>
       <c r="D29" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E29" t="s">
-        <v>52</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30">
         <v>8</v>
       </c>
-      <c r="B30" t="s">
-        <v>53</v>
-      </c>
-      <c r="C30" s="1">
-        <v>17</v>
-      </c>
       <c r="D30" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E30" t="s">
-        <v>52</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>12</v>
-      </c>
-      <c r="C31" s="1">
-        <v>22</v>
+        <v>43</v>
+      </c>
+      <c r="C31">
+        <v>25</v>
       </c>
       <c r="D31" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E31" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="1">
-        <v>12</v>
+        <v>44</v>
+      </c>
+      <c r="C32">
+        <v>65</v>
       </c>
       <c r="D32" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E32" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" s="1">
+        <v>45</v>
+      </c>
+      <c r="C33">
         <v>85</v>
       </c>
       <c r="D33" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E33" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>55</v>
-      </c>
-      <c r="C34" s="1">
-        <v>35</v>
+        <v>46</v>
+      </c>
+      <c r="C34">
+        <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E34" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>56</v>
-      </c>
-      <c r="C35" s="1">
-        <v>120</v>
+        <v>47</v>
+      </c>
+      <c r="C35">
+        <v>15</v>
       </c>
       <c r="D35" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E35" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>57</v>
-      </c>
-      <c r="C36" s="1">
-        <v>160</v>
+        <v>48</v>
+      </c>
+      <c r="C36">
+        <v>5</v>
       </c>
       <c r="D36" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E36" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>59</v>
-      </c>
-      <c r="C37" s="1">
-        <v>2.8</v>
+        <v>49</v>
+      </c>
+      <c r="C37">
+        <v>18</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E37" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>60</v>
-      </c>
-      <c r="C38" s="1">
-        <v>55</v>
+        <v>50</v>
+      </c>
+      <c r="C38">
+        <v>45</v>
       </c>
       <c r="D38" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>61</v>
-      </c>
-      <c r="C39" s="1">
-        <v>75</v>
+        <v>51</v>
+      </c>
+      <c r="C39">
+        <v>120</v>
       </c>
       <c r="D39" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E39" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="B40" t="s">
-        <v>62</v>
-      </c>
-      <c r="C40" s="1">
-        <v>35</v>
+        <v>52</v>
+      </c>
+      <c r="C40">
+        <v>95</v>
       </c>
       <c r="D40" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E40" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
-      </c>
-      <c r="C41" s="1">
-        <v>180</v>
+        <v>53</v>
+      </c>
+      <c r="C41">
+        <v>120</v>
       </c>
       <c r="D41" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E41" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>64</v>
-      </c>
-      <c r="C42" s="1">
-        <v>22</v>
+        <v>54</v>
+      </c>
+      <c r="C42">
+        <v>180</v>
       </c>
       <c r="D42" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E42" t="s">
-        <v>52</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>29</v>
-      </c>
-      <c r="C43" s="1">
-        <v>28</v>
+        <v>55</v>
+      </c>
+      <c r="C43">
+        <v>280</v>
       </c>
       <c r="D43" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E43" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>31</v>
-      </c>
-      <c r="C44" s="1">
-        <v>65</v>
+        <v>56</v>
+      </c>
+      <c r="C44">
+        <v>420</v>
       </c>
       <c r="D44" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E44" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>32</v>
-      </c>
-      <c r="C45" s="1">
-        <v>30</v>
+        <v>57</v>
+      </c>
+      <c r="C45">
+        <v>6</v>
       </c>
       <c r="D45" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E45" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B46" t="s">
-        <v>65</v>
-      </c>
-      <c r="C46" s="1">
-        <v>12</v>
+        <v>58</v>
+      </c>
+      <c r="C46">
+        <v>9</v>
       </c>
       <c r="D46" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E46" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
-        <v>67</v>
-      </c>
-      <c r="C47" s="1">
-        <v>45</v>
+        <v>59</v>
+      </c>
+      <c r="C47">
+        <v>18</v>
       </c>
       <c r="D47" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E47" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>68</v>
-      </c>
-      <c r="C48" s="1">
-        <v>65</v>
+        <v>60</v>
+      </c>
+      <c r="C48">
+        <v>18</v>
       </c>
       <c r="D48" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E48" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B49" t="s">
-        <v>69</v>
-      </c>
-      <c r="C49" s="1">
-        <v>85</v>
+        <v>15</v>
+      </c>
+      <c r="C49">
+        <v>20</v>
       </c>
       <c r="D49" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E49" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B50" t="s">
-        <v>70</v>
-      </c>
-      <c r="C50" s="1">
-        <v>120</v>
+        <v>61</v>
+      </c>
+      <c r="C50">
+        <v>25</v>
       </c>
       <c r="D50" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E50" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B51" t="s">
-        <v>71</v>
-      </c>
-      <c r="C51" s="1">
-        <v>180</v>
+        <v>62</v>
+      </c>
+      <c r="C51">
+        <v>35</v>
       </c>
       <c r="D51" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E51" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B52" t="s">
-        <v>72</v>
-      </c>
-      <c r="C52" s="1">
-        <v>220</v>
+        <v>63</v>
+      </c>
+      <c r="C52">
+        <v>85</v>
       </c>
       <c r="D52" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E52" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B53" t="s">
-        <v>73</v>
-      </c>
-      <c r="C53" s="1">
-        <v>95</v>
+        <v>64</v>
+      </c>
+      <c r="C53">
+        <v>140</v>
       </c>
       <c r="D53" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E53" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B54" t="s">
-        <v>74</v>
-      </c>
-      <c r="C54" s="1">
-        <v>110</v>
+        <v>16</v>
+      </c>
+      <c r="C54">
+        <v>8</v>
       </c>
       <c r="D54" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E54" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>75</v>
-      </c>
-      <c r="C55" s="1">
-        <v>75</v>
+        <v>65</v>
+      </c>
+      <c r="C55">
+        <v>12</v>
       </c>
       <c r="D55" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E55" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B56" t="s">
-        <v>76</v>
-      </c>
-      <c r="C56" s="1">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="C56">
+        <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E56" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B57" t="s">
-        <v>77</v>
-      </c>
-      <c r="C57" s="1">
-        <v>8</v>
+        <v>66</v>
+      </c>
+      <c r="C57">
+        <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E57" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B58" t="s">
-        <v>78</v>
-      </c>
-      <c r="C58" s="1">
-        <v>15</v>
+        <v>67</v>
+      </c>
+      <c r="C58">
+        <v>14</v>
       </c>
       <c r="D58" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E58" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -1688,16 +1648,16 @@
         <v>14</v>
       </c>
       <c r="B59" t="s">
-        <v>15</v>
-      </c>
-      <c r="C59" s="1">
-        <v>18</v>
+        <v>68</v>
+      </c>
+      <c r="C59">
+        <v>3</v>
       </c>
       <c r="D59" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E59" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -1705,16 +1665,16 @@
         <v>14</v>
       </c>
       <c r="B60" t="s">
-        <v>79</v>
-      </c>
-      <c r="C60" s="1">
-        <v>22</v>
+        <v>69</v>
+      </c>
+      <c r="C60">
+        <v>5</v>
       </c>
       <c r="D60" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E60" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -1722,16 +1682,16 @@
         <v>14</v>
       </c>
       <c r="B61" t="s">
-        <v>80</v>
-      </c>
-      <c r="C61" s="1">
-        <v>22</v>
+        <v>70</v>
+      </c>
+      <c r="C61">
+        <v>7</v>
       </c>
       <c r="D61" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E61" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -1739,16 +1699,16 @@
         <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>16</v>
-      </c>
-      <c r="C62" s="1">
-        <v>320</v>
+        <v>71</v>
+      </c>
+      <c r="C62">
+        <v>6</v>
       </c>
       <c r="D62" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E62" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1756,16 +1716,16 @@
         <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>81</v>
-      </c>
-      <c r="C63" s="1">
-        <v>45</v>
+        <v>18</v>
+      </c>
+      <c r="C63">
+        <v>8</v>
       </c>
       <c r="D63" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E63" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -1773,271 +1733,305 @@
         <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>82</v>
-      </c>
-      <c r="C64" s="1">
-        <v>120</v>
+        <v>72</v>
+      </c>
+      <c r="C64">
+        <v>10</v>
       </c>
       <c r="D64" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E64" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B65" t="s">
-        <v>84</v>
-      </c>
-      <c r="C65" s="1">
-        <v>180</v>
+        <v>73</v>
+      </c>
+      <c r="C65">
+        <v>15</v>
       </c>
       <c r="D65" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E65" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B66" t="s">
-        <v>85</v>
-      </c>
-      <c r="C66" s="1">
-        <v>280</v>
+        <v>74</v>
+      </c>
+      <c r="C66">
+        <v>65</v>
       </c>
       <c r="D66" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E66" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B67" t="s">
-        <v>86</v>
-      </c>
-      <c r="C67" s="1">
-        <v>20</v>
+        <v>75</v>
+      </c>
+      <c r="C67">
+        <v>120</v>
       </c>
       <c r="D67" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E67" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B68" t="s">
-        <v>87</v>
-      </c>
-      <c r="C68" s="1">
-        <v>8</v>
+        <v>76</v>
+      </c>
+      <c r="C68">
+        <v>4</v>
       </c>
       <c r="D68" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E68" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>88</v>
-      </c>
-      <c r="C69" s="1">
-        <v>7</v>
+        <v>77</v>
+      </c>
+      <c r="C69">
+        <v>25</v>
       </c>
       <c r="D69" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E69" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B70" t="s">
-        <v>89</v>
-      </c>
-      <c r="C70" s="1">
-        <v>8</v>
+        <v>78</v>
+      </c>
+      <c r="C70">
+        <v>45</v>
       </c>
       <c r="D70" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E70" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B71" t="s">
-        <v>90</v>
-      </c>
-      <c r="C71" s="1">
-        <v>85</v>
+        <v>79</v>
+      </c>
+      <c r="C71">
+        <v>6</v>
       </c>
       <c r="D71" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E71" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B72" t="s">
-        <v>92</v>
-      </c>
-      <c r="C72" s="1">
-        <v>45</v>
+        <v>80</v>
+      </c>
+      <c r="C72">
+        <v>18</v>
       </c>
       <c r="D72" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E72" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B73" t="s">
-        <v>93</v>
-      </c>
-      <c r="C73" s="1">
-        <v>55</v>
+        <v>81</v>
+      </c>
+      <c r="C73">
+        <v>3</v>
       </c>
       <c r="D73" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E73" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B74" t="s">
-        <v>94</v>
-      </c>
-      <c r="C74" s="1">
-        <v>25</v>
+        <v>82</v>
+      </c>
+      <c r="C74">
+        <v>5</v>
       </c>
       <c r="D74" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E74" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B75" t="s">
-        <v>95</v>
-      </c>
-      <c r="C75" s="1">
-        <v>35</v>
+        <v>83</v>
+      </c>
+      <c r="C75">
+        <v>12</v>
       </c>
       <c r="D75" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E75" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
-        <v>96</v>
-      </c>
-      <c r="C76" s="1">
-        <v>22</v>
+        <v>84</v>
+      </c>
+      <c r="C76">
+        <v>15</v>
       </c>
       <c r="D76" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E76" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
-        <v>97</v>
-      </c>
-      <c r="C77" s="1">
-        <v>65</v>
+        <v>85</v>
+      </c>
+      <c r="C77">
+        <v>4</v>
       </c>
       <c r="D77" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E77" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B78" t="s">
-        <v>98</v>
-      </c>
-      <c r="C78" s="1">
+        <v>86</v>
+      </c>
+      <c r="C78">
         <v>18</v>
       </c>
       <c r="D78" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E78" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
-        <v>99</v>
-      </c>
-      <c r="C79" s="1">
-        <v>280</v>
+        <v>87</v>
+      </c>
+      <c r="C79">
+        <v>35</v>
       </c>
       <c r="D79" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="E79" t="s">
-        <v>28</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>14</v>
+      </c>
+      <c r="B80" t="s">
+        <v>88</v>
+      </c>
+      <c r="C80">
+        <v>45</v>
+      </c>
+      <c r="D80" t="s">
+        <v>90</v>
+      </c>
+      <c r="E80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>14</v>
+      </c>
+      <c r="B81" t="s">
+        <v>89</v>
+      </c>
+      <c r="C81">
+        <v>120</v>
+      </c>
+      <c r="D81" t="s">
+        <v>90</v>
+      </c>
+      <c r="E81" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>